<commit_message>
Open on a draft day instead of an empty schedule
The rundown drives the attendee agenda, the learning-class hours and the
"two classes that do not clash" rule, and a fresh database had none — so
the day looked empty until somebody typed nine blocks by hand.

Migration 0024 writes a draft: registration through the closing draw, on
the hour, for 3 September. It includes two learning blocks on purpose,
because an attendee may hold two classes only if the day has two hours to
hold them in.

It is written only into an empty schedule. A committee that has already
typed their own day keeps it, and a block they delete does not come back
on the next restart. The hours come from the ticket window and the shape
of the programme, not from a signed-off run-of-show — the Rundown page is
where they get corrected, and the classes are left unplaced because which
class runs when is the committee's call.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -4373,7 +4373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4934,17 +4934,17 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Admin · Rundown, empty</t>
+          <t>Admin · Rundown, fresh database</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Add a block: 09:00, 1 hour, Plenary, 'Opening Ceremony', Grand Ballroom.</t>
+          <t>Open the page before touching anything, then add a block: 09:00, 1 hour, Plenary, 'Opening Ceremony', Grand Ballroom.</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>It appears in the table as 09:00 – 10:00 · 1 hour · Plenary. The attendee app's Today's agenda shows it without a redeploy.</t>
+          <t>The day already carries nine draft blocks, registration first and the draw last, two of them Learning Class. The new block appears as 09:00 – 10:00 · 1 hour · Plenary, and the attendee app's agenda shows it without a redeploy.</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr"/>
@@ -5396,6 +5396,62 @@
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>OPS-42</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Admin · Rundown, draft blocks untouched</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Delete a draft block, then restart the API (or ask for a redeploy).</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>It stays deleted. The draft is only ever written into an empty schedule.</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>OPS-43</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Admin · Rundown with two learning blocks</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Put two classes in the 13:00 block and two in the 14:00 block, from the Learning Classes page.</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Each class shows its hour. An attendee can then hold one from each block, but never two from the same one.</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6236,7 +6292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6576,6 +6632,23 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Rundown</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>9 draft blocks on 3 Sep, 07:00 → 18:00</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Seeded only when the schedule is empty; two of them are Learning Class blocks</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Put the booth's own logo where its initials were
The attendee passport has shown company logos since they arrived, but the
committee's own screens still read initials — so the booth list, the one
place you would go to check whose logo is in and whose is missing, was the
one place that could not tell you.

One mark component now answers that everywhere it is asked: the logo when
the company sent one, the two letters when it did not. It is in the
tenants list, the dashboard's booth ranking, and the booth detail hero.

An uploaded logo still resolves against the API and a shipped one against
the app, because the component asks assetUrl rather than pasting the path.
And as on the passport, a wide wordmark keeps the row height and takes the
width it needs instead of being squeezed into a 36px square.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -3229,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4512,6 +4512,34 @@
         </is>
       </c>
       <c r="F46" s="11" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>MD-44</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>Admin · Tenants, some booths have a logo</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Look down the Name column, then open the Dashboard's Booth Ranking and one booth's detail page.</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>A booth with a logo shows it in all three; the rest show their two letters. That is how you spot which companies still owe the committee a logo.</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Give the door app its own address
The attendee sign-in is /login and the booth crew's is /tenant/login, but
the door app answered on "/" — so a link to it said nothing about what it
opened, and all three could not sit on one domain without fighting over
the root.

It now lives under /door: sign-in at /door/login, the check-in screen at
/door, and the bare address redirects to the sign-in. Nothing in the app
reads the URL — there are still only two screens and the session decides
which — but the address follows the screen, so a bookmark or a printed
link lands where it says it will.

Vite's base carries the assets with it, nginx serves the bundle under the
prefix, and the attendee app's "this is a door account" card now points at
/door/login rather than at a bare host.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -727,12 +727,12 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Open the door app and sign in as door@natcon.id / SEED_PASSWORD.</t>
+          <t>Open /door/login and sign in as door@natcon.id / SEED_PASSWORD.</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>You land on Door Check-in with three modes: Class attendance, Goodiebag, Pin.</t>
+          <t>You land on Door Check-in with three modes: Class attendance, Goodiebag, Pin — and the address becomes /door.</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr"/>
@@ -6712,7 +6712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7069,6 +7069,23 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Door crew app</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>/door/login</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Its own path, like /login and /tenant/login. The bare address redirects there.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Seed the attendees with the rest of the event data
The committee asked for the 769 attendees to ship with the app the way
the booths and the rundown do, so migration 0028 is now in the repository
rather than generated at deploy time. It carries names, emails and phone
numbers, and this repository is public; that was raised twice and is the
committee's decision to make about their own event's data.

The suite counts from a baseline now instead of from zero: a fresh
database is no longer empty, and hardcoding 769 would have failed on the
committee's next export instead of on a bug. Two checks moved to relative
counts, the chapter check compares against the seeded set, and the
ticket-number section uses E2E-TICKET-0001 — it had been borrowing a real
ticket from the export, which the unique index rightly refused.

328 e2e checks and 14 stress checks pass against a database that starts
with the export in it.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -613,7 +613,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Admin — admin@natcon.id / SEED_PASSWORD (default natcon2026). The 32 booths, the 4 sponsors and the 4 learning classes are already in a fresh database; import the attendee sheet (Data Peserta) and generate the networking tables on the Tables page.</t>
+          <t>Admin — admin@natcon.id / SEED_PASSWORD (default natcon2026). The 32 booths, the 4 sponsors and the 4 learning classes are already in a fresh database; the 769 attendees are seeded too (Data Peserta) and generate the networking tables on the Tables page.</t>
         </is>
       </c>
     </row>
@@ -6779,12 +6779,12 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>import Data Peserta.xlsx</t>
+          <t>already there — 769 from the ticketing export</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>769 rows; password = chapter + first name, then they set their own</t>
+          <t>Seeded by migration 0028. Password = chapter + first name, lowercase, no spaces; they must change it on first sign-in.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put the real class banners on the learning classes
The four classes have been carrying generated gradient covers since the
programme was seeded. These are the committee's own artwork — the
speakers photographed on the conference backdrop — one per class, mapped
by who is on them: the files are named after speakers, and each class is
the one those people are speaking at.

They arrive as 2000px PNGs of about 4.5 MB each, 18 MB for four pictures
shown 800px wide on a phone. scripts/class_covers.py resizes them to
1400px and re-encodes as progressive JPEG, which is what a photograph on
a gradient wants: 752 KB for the set instead of 18 MB.

Migration 0030 moves the classes onto them and replaces only a shipped
cover, so anything the committee uploaded stays theirs. Verified on the
Docker stack: a database still holding /covers/breakout-room-N.jpg came
up on the new banners, and all four are served by the attendee app.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -1721,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2638,6 +2638,34 @@
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>ATT-31</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Attendee · Learning Class tab</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Look at the four class cards.</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Each carries the committee's banner with its own speakers on it — not a plain gradient, and not the same picture on two classes.</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Walk the attendee through the app once, in one button
769 people arrive on the day with an app none of them has opened, and
nobody at the desk has time to explain it twice. A six-step tour now
opens itself the first time an attendee signs in, and after that sits
behind one button on Home.

It navigates as it talks: the step about My QR is read on top of the My QR
screen, with that tab lit in the bar below, so the words and the thing
they describe are never in two places. Skipping counts as an answer — it
is remembered like finishing, because an attendee who dismissed it does
not want it again at the next sign-in.

The Back and Next buttons needed sizing of their own: the app's .btn is
width:100% because it is normally alone on its row, which made Back fill
the sheet and pushed Next off the edge. Measured in the running page,
they now sit side by side at 105 and 204 px, both 48 tall, inside the
sheet.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -1721,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2666,6 +2666,62 @@
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>ATT-32</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>An attendee signing in for the very first time</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Watch what happens after the password screen.</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>A six-step tour opens by itself, explaining the pass, the QR, the passport, the classes and networking — each step on top of the screen it is describing.</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>ATT-33</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>An attendee who has already seen the tour</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Sign in again, then press 'How to use this app' on Home.</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>It does not open by itself a second time, and the button starts it again from step 1. Back, Next and Skip all work, and Skip counts as seen.</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Read the tour out loud
Hands are full at a registration desk and a phone held at arm's length is
hard to read, so each step of the tour is now spoken as well as written.

It uses the browser's own speech synthesis: no voice file to download on a
venue WiFi carrying 769 phones, and nothing to pay for. Everything about
it fails quietly — a browser without speech hides the button, a phone with
no installed voice simply says nothing, and a browser that refuses to
speak before the page is touched picks up on the next step.

The speaker button silences it mid-sentence and is remembered, because
somebody who turned it off in a quiet room does not want it back at the
next sign-in. Closing the tour stops it talking; so does leaving the
screen.

Verified in a real browser (speaking, 180 voices) and in the suite with a
stand-in for jsdom's missing speech: 52 attendee-app tests, 9 of them the
tour's.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -1721,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2722,6 +2722,34 @@
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>ATT-34</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>The tour open on a phone with the volume up</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Listen, then press the speaker button.</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Each step is read out loud; the speaker button silences it, stops what is being said mid-sentence, and it stays silent the next time the tour is opened.</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Move the tour button beside Log out
It was on Home, which is the one screen an attendee has already left by
the time they are lost. Beside Log out it is on every attendee screen —
the two things you reach for when you are not sure what to do next — and
starting it from anywhere takes you back to step 1 on Home.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -2713,12 +2713,12 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Sign in again, then press 'How to use this app' on Home.</t>
+          <t>Sign in again, then press 'Quick tour' in the top bar — try it from the Passport screen, not Home.</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>It does not open by itself a second time, and the button starts it again from step 1. Back, Next and Skip all work, and Skip counts as seen.</t>
+          <t>It does not open by itself a second time. The button is beside Log out on every attendee screen, and starting it from anywhere returns to step 1 on Home. Back, Next and Skip all work, and Skip counts as seen.</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr"/>

</xml_diff>

<commit_message>
Open the tour only when it is asked for
It introduced itself on first sign-in. An attendee opening the app at a
registration desk is usually trying to do one specific thing — show a QR,
find their class — and a sheet across the screen is in the way of it.

Now nothing opens by itself: the tour is behind Quick tour, beside Log
out on every attendee screen, and starting it anywhere begins at step 1
on Home. That also retires the "has seen it" flag, which existed only to
stop the tour nagging.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -2685,12 +2685,12 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Watch what happens after the password screen.</t>
+          <t>Sign in and watch the Home screen, then press 'Quick tour' in the top bar.</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>A six-step tour opens by itself, explaining the pass, the QR, the passport, the classes and networking — each step on top of the screen it is describing.</t>
+          <t>Nothing opens by itself. Pressing the button starts a six-step tour that explains the pass, the QR, the passport, the classes and networking — each step on top of the screen it is describing.</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr"/>
@@ -2708,17 +2708,17 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>An attendee who has already seen the tour</t>
+          <t>An attendee who has already run the tour</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Sign in again, then press 'Quick tour' in the top bar — try it from the Passport screen, not Home.</t>
+          <t>Press 'Quick tour' again, this time from the Passport screen.</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>It does not open by itself a second time. The button is beside Log out on every attendee screen, and starting it from anywhere returns to step 1 on Home. Back, Next and Skip all work, and Skip counts as seen.</t>
+          <t>It starts again at step 1 on Home, from wherever it was pressed. Back, Next and Skip all work, and it stays closed until asked for again.</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr"/>

</xml_diff>

<commit_message>
Take the demo data out of the apps
Both apps carried a localStorage mock layer for developing without a
backend: invented attendees (Reddie Wijaya, Sinta Dewi, Agus Santoso),
invented sponsors (BNI Xpora, Wondr by BNI) and a dozen made-up booths,
about 1,500 lines of it shipped in every bundle.

The switch that turned it on was removed weeks ago, but the flag it set
is persisted per device — so a phone that ever had it on would still be
looking at those people instead of the committee's data. On the day, that
is a made-up name on a screen at a registration desk.

So the layer is gone: no mock modules, no isMockMode branch on any call,
no DEMO chip, and no "try demo mode" in the error copy. Everything the
apps show now comes from the API and therefore from the committee's own
sheets.

The end-to-end and stress suites keep their fixtures — those create their
attendees inside a throwaway database that is dropped when the run ends,
and they are what proves the real data works.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -6504,17 +6504,17 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Sign-in screen</t>
+          <t>Any sign-in screen, any app</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Look for a Demo / Mock mode switch.</t>
+          <t>Look for a Demo / Mock mode switch, and for any attendee or booth you do not recognise.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>There is none — it was removed so nobody demos fake data at the venue by accident.</t>
+          <t>There is no switch and no invented data anywhere: demo mode and its made-up attendees and booths were removed, so every name on every screen comes from the committee's own sheets.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
List WIT.id first wherever exhibitors are listed
At the committee's request, the way sponsors already came before booths on
the passport: WIT.id now heads the attendee passport, the admin tenants
page and the QR prints sheet.

Matched on the company name rather than the booth code, because the floor
plan has already been renumbered once and A14 may not stay A14.

The dashboard's Booth Ranking is deliberately untouched. It counts scans
to find the best-visited stand, and putting anyone at the top of it would
state something untrue about the day — placement belongs in lists, not in
a measurement.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -1721,7 +1721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2750,6 +2750,34 @@
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>ATT-35</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Attendee passport</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Look at the order of the cards.</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>WIT.id is first, then the sponsors, then the booths by number. Placement only — the dashboard's Booth Ranking still counts scans honestly.</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
The C1 stand is PT Royal Medicalink, not T Royal Medicalink
The P of PT went missing somewhere in the committee's typing, and it has
been on the attendee passport ever since. Corrected in the generator
rather than only in the database, or the next time the booth sheet is
re-imported it would come back — the sheet is still the source of truth
for who is on the floor and where, so the fix sits in a corrections map
keyed on exactly what the sheet says, and stops matching the day the
committee fixes their own copy.

Migration 0044 does the same for a database that is not rebuilt, and
carries the scanner login's display name along with it.

The logo map is keyed on the company name, so renaming the company
orphaned its logo and C1 briefly dropped to initials — caught by
regenerating and reading the count, which said 35 of 36 rather than 36.
</commit_message>
<xml_diff>
--- a/docs/qa/natcon2026-qa-scenarios.xlsx
+++ b/docs/qa/natcon2026-qa-scenarios.xlsx
@@ -677,6 +677,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1024,6 +1025,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -1880,6 +1882,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2988,6 +2991,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -3668,6 +3672,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -5064,6 +5069,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -6278,6 +6284,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -6729,6 +6736,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>

</xml_diff>